<commit_message>
DP: create_forecast_basic - utils - monitoring_df.ipynb - aprt division total_emp
</commit_message>
<xml_diff>
--- a/create_forecast_basic/utils/monitoring_df_fixed_1.xlsx
+++ b/create_forecast_basic/utils/monitoring_df_fixed_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1529" uniqueCount="1509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="1523">
   <si>
     <t>2020</t>
   </si>
@@ -244,22 +244,22 @@
     <t>percentage growth arabs_behined_seperation_wall 2045-2050</t>
   </si>
   <si>
-    <t>percentage growth U_Orthodox age15_24 2020-2025</t>
-  </si>
-  <si>
-    <t>percentage growth U_Orthodox age15_24 2025-2030</t>
-  </si>
-  <si>
-    <t>percentage growth U_Orthodox age15_24 2030-2035</t>
-  </si>
-  <si>
-    <t>percentage growth U_Orthodox age15_24 2035-2040</t>
-  </si>
-  <si>
-    <t>percentage growth U_Orthodox age15_24 2040-2045</t>
-  </si>
-  <si>
-    <t>percentage growth U_Orthodox age15_24 2045-2050</t>
+    <t>percentage growth U_Orthodox age18_24 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth U_Orthodox age18_24 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth U_Orthodox age18_24 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth U_Orthodox age18_24 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth U_Orthodox age18_24 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth U_Orthodox age18_24 2045-2050</t>
   </si>
   <si>
     <t>percentage growth Arab age20_29 2020-2025</t>
@@ -3166,31 +3166,31 @@
     <t>emp_okev at הר אדר in 2050</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3236,31 +3236,31 @@
     <t>emp_okev at מבשרת ציון in 2050</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3411,31 +3411,31 @@
     <t>emp_okev at עמנואל in 2050</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3817,31 +3817,31 @@
     <t>total_emp at הר אדר in 2050</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3887,31 +3887,31 @@
     <t>total_emp at מבשרת ציון in 2050</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -4062,31 +4062,31 @@
     <t>total_emp at עמנואל in 2050</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -4529,6 +4529,48 @@
   </si>
   <si>
     <t>pop division emp_okev at תלפיות מזרח in 2025</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2020</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2025</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2030</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2035</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2040</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2045</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2050</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2020</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2025</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2030</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2035</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2040</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2045</t>
+  </si>
+  <si>
+    <t>aprt division total_emp in 2050</t>
   </si>
   <si>
     <t>1,758,461</t>
@@ -4940,7 +4982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1488"/>
+  <dimension ref="A1:E1502"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4962,16 +5004,16 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>1491</v>
+        <v>1505</v>
       </c>
       <c r="C2" t="s">
-        <v>1491</v>
+        <v>1505</v>
       </c>
       <c r="D2" t="s">
-        <v>1491</v>
+        <v>1505</v>
       </c>
       <c r="E2" t="s">
-        <v>1491</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -4979,13 +5021,13 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>1496</v>
+        <v>1510</v>
       </c>
       <c r="D3" t="s">
-        <v>1501</v>
+        <v>1515</v>
       </c>
       <c r="E3" t="s">
-        <v>1505</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4993,16 +5035,16 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>1492</v>
+        <v>1506</v>
       </c>
       <c r="C4" t="s">
-        <v>1492</v>
+        <v>1506</v>
       </c>
       <c r="D4" t="s">
-        <v>1492</v>
+        <v>1506</v>
       </c>
       <c r="E4" t="s">
-        <v>1492</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -5010,13 +5052,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>1497</v>
+        <v>1511</v>
       </c>
       <c r="D5" t="s">
-        <v>1502</v>
+        <v>1516</v>
       </c>
       <c r="E5" t="s">
-        <v>1506</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5109,16 +5151,16 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
       <c r="C11" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
       <c r="D11" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
       <c r="E11" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -5126,13 +5168,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
       <c r="D12" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
       <c r="E12" t="s">
-        <v>1493</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -5140,16 +5182,16 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>1494</v>
+        <v>1508</v>
       </c>
       <c r="C13" t="s">
-        <v>1494</v>
+        <v>1508</v>
       </c>
       <c r="D13" t="s">
-        <v>1494</v>
+        <v>1508</v>
       </c>
       <c r="E13" t="s">
-        <v>1494</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -5157,13 +5199,13 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>1498</v>
+        <v>1512</v>
       </c>
       <c r="D14" t="s">
-        <v>1503</v>
+        <v>1517</v>
       </c>
       <c r="E14" t="s">
-        <v>1507</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -5171,16 +5213,16 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>1495</v>
+        <v>1509</v>
       </c>
       <c r="C15" t="s">
-        <v>1495</v>
+        <v>1509</v>
       </c>
       <c r="D15" t="s">
-        <v>1495</v>
+        <v>1509</v>
       </c>
       <c r="E15" t="s">
-        <v>1495</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -5188,13 +5230,13 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>1499</v>
+        <v>1513</v>
       </c>
       <c r="D16" t="s">
-        <v>1504</v>
+        <v>1518</v>
       </c>
       <c r="E16" t="s">
-        <v>1508</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -5355,10 +5397,10 @@
         <v>28</v>
       </c>
       <c r="C26">
-        <v>188.1410644079084</v>
+        <v>188.1410644079083</v>
       </c>
       <c r="D26">
-        <v>183.9696620191286</v>
+        <v>183.9696620191285</v>
       </c>
       <c r="E26">
         <v>185.6774324006336</v>
@@ -5635,13 +5677,13 @@
         <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>1500</v>
+        <v>1514</v>
       </c>
       <c r="D46" t="s">
-        <v>1500</v>
+        <v>1514</v>
       </c>
       <c r="E46" t="s">
-        <v>1500</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -6027,13 +6069,13 @@
         <v>76</v>
       </c>
       <c r="C74">
-        <v>42.09690954865545</v>
+        <v>41.54781713017986</v>
       </c>
       <c r="D74">
-        <v>40.43492538402597</v>
+        <v>37.86546232469693</v>
       </c>
       <c r="E74">
-        <v>43.61020907067537</v>
+        <v>41.29394131473998</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -6041,13 +6083,13 @@
         <v>77</v>
       </c>
       <c r="C75">
-        <v>15.77758091643236</v>
+        <v>16.20276428907952</v>
       </c>
       <c r="D75">
-        <v>12.02811192808335</v>
+        <v>11.45833333333333</v>
       </c>
       <c r="E75">
-        <v>15.17559404714267</v>
+        <v>14.76593805857682</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -6055,13 +6097,13 @@
         <v>78</v>
       </c>
       <c r="C76">
-        <v>14.69593470691299</v>
+        <v>14.92200295449436</v>
       </c>
       <c r="D76">
-        <v>17.6768672379605</v>
+        <v>15.38038457406811</v>
       </c>
       <c r="E76">
-        <v>20.61501469704239</v>
+        <v>18.26719681746647</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -6069,13 +6111,13 @@
         <v>79</v>
       </c>
       <c r="C77">
-        <v>9.364742508254336</v>
+        <v>9.228582057359025</v>
       </c>
       <c r="D77">
-        <v>16.96278121027581</v>
+        <v>18.89400750040033</v>
       </c>
       <c r="E77">
-        <v>21.28160577934251</v>
+        <v>22.99735241157777</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -6083,13 +6125,13 @@
         <v>80</v>
       </c>
       <c r="C78">
-        <v>18.44823699460291</v>
+        <v>22.02142917674674</v>
       </c>
       <c r="D78">
-        <v>14.17119507982644</v>
+        <v>14.86172408716597</v>
       </c>
       <c r="E78">
-        <v>18.17684869276734</v>
+        <v>18.55999798460181</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -6097,13 +6139,13 @@
         <v>81</v>
       </c>
       <c r="C79">
-        <v>6.347749179942457</v>
+        <v>6.722550328710719</v>
       </c>
       <c r="D79">
-        <v>12.19823562618298</v>
+        <v>12.95406729488314</v>
       </c>
       <c r="E79">
-        <v>16.27268957156985</v>
+        <v>16.97984913411482</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -25830,6 +25872,202 @@
       </c>
       <c r="E1488">
         <v>5.208887551814326</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:5">
+      <c r="A1489" s="1" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C1489">
+        <v>0.274510590027404</v>
+      </c>
+      <c r="D1489">
+        <v>0.274510590027404</v>
+      </c>
+      <c r="E1489">
+        <v>0.274510590027404</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:5">
+      <c r="A1490" s="1" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C1490">
+        <v>0.1085610779961064</v>
+      </c>
+      <c r="D1490">
+        <v>0.1042627101407602</v>
+      </c>
+      <c r="E1490">
+        <v>0.1051127003854925</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:5">
+      <c r="A1491" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C1491">
+        <v>0.1125054369322683</v>
+      </c>
+      <c r="D1491">
+        <v>0.1060000485240958</v>
+      </c>
+      <c r="E1491">
+        <v>0.108259127712942</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:5">
+      <c r="A1492" s="1" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C1492">
+        <v>0.117776582480796</v>
+      </c>
+      <c r="D1492">
+        <v>0.1088794149716449</v>
+      </c>
+      <c r="E1492">
+        <v>0.1124915624920027</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:5">
+      <c r="A1493" s="1" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C1493">
+        <v>0.1227534623323177</v>
+      </c>
+      <c r="D1493">
+        <v>0.1111431609688907</v>
+      </c>
+      <c r="E1493">
+        <v>0.1165598777550276</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:5">
+      <c r="A1494" s="1" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C1494">
+        <v>0.1292444792424143</v>
+      </c>
+      <c r="D1494">
+        <v>0.1129801244081925</v>
+      </c>
+      <c r="E1494">
+        <v>0.1202497001616002</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:5">
+      <c r="A1495" s="1" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C1495">
+        <v>0.1309869731098417</v>
+      </c>
+      <c r="D1495">
+        <v>0.1150036371136272</v>
+      </c>
+      <c r="E1495">
+        <v>0.1240135292494374</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:5">
+      <c r="A1496" s="1" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C1496">
+        <v>1.114079232346069</v>
+      </c>
+      <c r="D1496">
+        <v>1.114079232346069</v>
+      </c>
+      <c r="E1496">
+        <v>1.114079232346069</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:5">
+      <c r="A1497" s="1" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C1497">
+        <v>1.159182665523671</v>
+      </c>
+      <c r="D1497">
+        <v>1.144472910686225</v>
+      </c>
+      <c r="E1497">
+        <v>1.14517662824113</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:5">
+      <c r="A1498" s="1" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C1498">
+        <v>1.188754352991139</v>
+      </c>
+      <c r="D1498">
+        <v>1.173077736396925</v>
+      </c>
+      <c r="E1498">
+        <v>1.174263741817146</v>
+      </c>
+    </row>
+    <row r="1499" spans="1:5">
+      <c r="A1499" s="1" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C1499">
+        <v>1.218643112621387</v>
+      </c>
+      <c r="D1499">
+        <v>1.206558686088572</v>
+      </c>
+      <c r="E1499">
+        <v>1.208720333611625</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:5">
+      <c r="A1500" s="1" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C1500">
+        <v>1.243413157309403</v>
+      </c>
+      <c r="D1500">
+        <v>1.23518656648838</v>
+      </c>
+      <c r="E1500">
+        <v>1.239806494952869</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:5">
+      <c r="A1501" s="1" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C1501">
+        <v>1.300436413012383</v>
+      </c>
+      <c r="D1501">
+        <v>1.252104471481292</v>
+      </c>
+      <c r="E1501">
+        <v>1.263459048274382</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:5">
+      <c r="A1502" s="1" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C1502">
+        <v>1.329352210290853</v>
+      </c>
+      <c r="D1502">
+        <v>1.275333581933721</v>
+      </c>
+      <c r="E1502">
+        <v>1.291052166578559</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DP: create_forecast_basic - utils - monitoring_df.ipynb - percentage growth emp education by Muni_Heb
</commit_message>
<xml_diff>
--- a/create_forecast_basic/utils/monitoring_df_fixed_1.xlsx
+++ b/create_forecast_basic/utils/monitoring_df_fixed_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1891" uniqueCount="1859">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="2033">
   <si>
     <t>2020</t>
   </si>
@@ -5579,6 +5579,546 @@
   </si>
   <si>
     <t>percentage growth emp education תלפיות מזרח 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2020-2025</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2025-2030</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2030-2035</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2035-2040</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2040-2045</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אבו גוש 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אורנית 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אלפי מנשה 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אפרת 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education אריאל 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אל 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית אריה-עופרים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education בית שמש 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ביתר עילית 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גבעת זאב 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education גוש עציון 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר אדר 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education הר חברון_x005F_x000D_
+ 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ירושלים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מבשרת ציון 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מגילות ים המלח_x005F_x000D_
+ 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין - מכבים - רעות 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מודיעין עילית 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה בנימין 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מטה יהודה 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אדומים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education מעלה אפרים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education עמנואל 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education ערבות הירדן_x005F_x000D_
+ 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קדומים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קריית ארבע 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרית יערים 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education קרני שומרון 2045-2050</t>
+  </si>
+  <si>
+    <t>percentage growth emp education שומרון 2045-2050</t>
   </si>
   <si>
     <t>1,758,461</t>
@@ -5990,7 +6530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1838"/>
+  <dimension ref="A1:E2012"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -6012,16 +6552,16 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>1841</v>
+        <v>2015</v>
       </c>
       <c r="C2" t="s">
-        <v>1841</v>
+        <v>2015</v>
       </c>
       <c r="D2" t="s">
-        <v>1841</v>
+        <v>2015</v>
       </c>
       <c r="E2" t="s">
-        <v>1841</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -6029,13 +6569,13 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>1846</v>
+        <v>2020</v>
       </c>
       <c r="D3" t="s">
-        <v>1851</v>
+        <v>2025</v>
       </c>
       <c r="E3" t="s">
-        <v>1855</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -6043,16 +6583,16 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>1842</v>
+        <v>2016</v>
       </c>
       <c r="C4" t="s">
-        <v>1842</v>
+        <v>2016</v>
       </c>
       <c r="D4" t="s">
-        <v>1842</v>
+        <v>2016</v>
       </c>
       <c r="E4" t="s">
-        <v>1842</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -6060,13 +6600,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>1847</v>
+        <v>2021</v>
       </c>
       <c r="D5" t="s">
-        <v>1852</v>
+        <v>2026</v>
       </c>
       <c r="E5" t="s">
-        <v>1856</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -6159,16 +6699,16 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
       <c r="C11" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
       <c r="D11" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
       <c r="E11" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -6176,13 +6716,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
       <c r="D12" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
       <c r="E12" t="s">
-        <v>1843</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -6190,16 +6730,16 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>1844</v>
+        <v>2018</v>
       </c>
       <c r="C13" t="s">
-        <v>1844</v>
+        <v>2018</v>
       </c>
       <c r="D13" t="s">
-        <v>1844</v>
+        <v>2018</v>
       </c>
       <c r="E13" t="s">
-        <v>1844</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -6207,13 +6747,13 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>1848</v>
+        <v>2022</v>
       </c>
       <c r="D14" t="s">
-        <v>1853</v>
+        <v>2027</v>
       </c>
       <c r="E14" t="s">
-        <v>1857</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -6221,16 +6761,16 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>1845</v>
+        <v>2019</v>
       </c>
       <c r="C15" t="s">
-        <v>1845</v>
+        <v>2019</v>
       </c>
       <c r="D15" t="s">
-        <v>1845</v>
+        <v>2019</v>
       </c>
       <c r="E15" t="s">
-        <v>1845</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -6238,13 +6778,13 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>1849</v>
+        <v>2023</v>
       </c>
       <c r="D16" t="s">
-        <v>1854</v>
+        <v>2028</v>
       </c>
       <c r="E16" t="s">
-        <v>1858</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -6685,13 +7225,13 @@
         <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="D46" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="E46" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -27083,13 +27623,13 @@
         <v>1505</v>
       </c>
       <c r="C1503">
-        <v>-26.68354606628418</v>
+        <v>-16.85929489135742</v>
       </c>
       <c r="D1503">
-        <v>-28.10066604614258</v>
+        <v>-17.64156723022461</v>
       </c>
       <c r="E1503">
-        <v>-26.38949012756348</v>
+        <v>-15.83106994628906</v>
       </c>
     </row>
     <row r="1504" spans="1:5">
@@ -27359,13 +27899,13 @@
         <v>1526</v>
       </c>
       <c r="C1524" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="D1524" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="E1524" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1525" spans="1:5">
@@ -27831,13 +28371,13 @@
         <v>1561</v>
       </c>
       <c r="C1559">
-        <v>22.70803070068359</v>
+        <v>4.33017110824585</v>
       </c>
       <c r="D1559">
-        <v>9.348258972167969</v>
+        <v>0.8684369325637817</v>
       </c>
       <c r="E1559">
-        <v>18.4731616973877</v>
+        <v>1.681298136711121</v>
       </c>
     </row>
     <row r="1560" spans="1:5">
@@ -27943,13 +28483,13 @@
         <v>1569</v>
       </c>
       <c r="C1567" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="D1567" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="E1567" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1568" spans="1:5">
@@ -28588,13 +29128,13 @@
         <v>1617</v>
       </c>
       <c r="C1615">
-        <v>15.13704109191895</v>
+        <v>3.691997051239014</v>
       </c>
       <c r="D1615">
-        <v>16.02740478515625</v>
+        <v>0.5136735439300537</v>
       </c>
       <c r="E1615">
-        <v>14.33720111846924</v>
+        <v>0.6098133325576782</v>
       </c>
     </row>
     <row r="1616" spans="1:5">
@@ -28840,13 +29380,13 @@
         <v>1635</v>
       </c>
       <c r="C1633" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="D1633" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="E1633" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1634" spans="1:5">
@@ -29223,7 +29763,7 @@
         <v>1663</v>
       </c>
       <c r="C1661" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1662" spans="1:5">
@@ -29357,13 +29897,13 @@
         <v>1673</v>
       </c>
       <c r="C1671">
-        <v>13.68764114379883</v>
+        <v>5.889151573181152</v>
       </c>
       <c r="D1671">
-        <v>15.86247730255127</v>
+        <v>0.5769818425178528</v>
       </c>
       <c r="E1671">
-        <v>18.48310661315918</v>
+        <v>1.787942409515381</v>
       </c>
     </row>
     <row r="1672" spans="1:5">
@@ -30126,13 +30666,13 @@
         <v>1729</v>
       </c>
       <c r="C1727">
-        <v>0.8824127912521362</v>
+        <v>0.6130074858665466</v>
       </c>
       <c r="D1727">
-        <v>2.5003662109375</v>
+        <v>0.5606398582458496</v>
       </c>
       <c r="E1727">
-        <v>9.929659843444824</v>
+        <v>0.7679650187492371</v>
       </c>
     </row>
     <row r="1728" spans="1:5">
@@ -30728,10 +31268,10 @@
         <v>1772</v>
       </c>
       <c r="C1770" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
       <c r="E1770" t="s">
-        <v>1850</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1771" spans="1:5">
@@ -30901,13 +31441,13 @@
         <v>1785</v>
       </c>
       <c r="C1783">
-        <v>6.790185451507568</v>
+        <v>0.2484400272369385</v>
       </c>
       <c r="D1783">
-        <v>11.82536602020264</v>
+        <v>0.5473768711090088</v>
       </c>
       <c r="E1783">
-        <v>10.5778923034668</v>
+        <v>1.028585910797119</v>
       </c>
     </row>
     <row r="1784" spans="1:5">
@@ -31669,6 +32209,2397 @@
       </c>
       <c r="E1838">
         <v>9.90286922454834</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:5">
+      <c r="A1839" s="1" t="s">
+        <v>1841</v>
+      </c>
+      <c r="C1839">
+        <v>-8.940157890319824</v>
+      </c>
+      <c r="D1839">
+        <v>-10.28324222564697</v>
+      </c>
+      <c r="E1839">
+        <v>-9.841169357299805</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:5">
+      <c r="A1840" s="1" t="s">
+        <v>1842</v>
+      </c>
+      <c r="C1840">
+        <v>-28.45031547546387</v>
+      </c>
+      <c r="D1840">
+        <v>-100</v>
+      </c>
+      <c r="E1840">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:5">
+      <c r="A1841" s="1" t="s">
+        <v>1843</v>
+      </c>
+      <c r="C1841">
+        <v>27.62912940979004</v>
+      </c>
+      <c r="D1841">
+        <v>28.98475074768066</v>
+      </c>
+      <c r="E1841">
+        <v>30.40701866149902</v>
+      </c>
+    </row>
+    <row r="1842" spans="1:5">
+      <c r="A1842" s="1" t="s">
+        <v>1844</v>
+      </c>
+      <c r="C1842">
+        <v>-97.96548461914062</v>
+      </c>
+      <c r="D1842">
+        <v>-97.9892578125</v>
+      </c>
+      <c r="E1842">
+        <v>-97.94863128662109</v>
+      </c>
+    </row>
+    <row r="1843" spans="1:5">
+      <c r="A1843" s="1" t="s">
+        <v>1845</v>
+      </c>
+      <c r="C1843">
+        <v>-25.80515670776367</v>
+      </c>
+      <c r="D1843">
+        <v>-25.80810546875</v>
+      </c>
+      <c r="E1843">
+        <v>-25.80306816101074</v>
+      </c>
+    </row>
+    <row r="1844" spans="1:5">
+      <c r="A1844" s="1" t="s">
+        <v>1846</v>
+      </c>
+      <c r="C1844">
+        <v>-92.50789642333984</v>
+      </c>
+      <c r="D1844">
+        <v>-92.59545135498047</v>
+      </c>
+      <c r="E1844">
+        <v>-92.44584655761719</v>
+      </c>
+    </row>
+    <row r="1845" spans="1:5">
+      <c r="A1845" s="1" t="s">
+        <v>1847</v>
+      </c>
+      <c r="C1845">
+        <v>45.0267219543457</v>
+      </c>
+      <c r="D1845">
+        <v>33.20018005371094</v>
+      </c>
+      <c r="E1845">
+        <v>48.18932342529297</v>
+      </c>
+    </row>
+    <row r="1846" spans="1:5">
+      <c r="A1846" s="1" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C1846">
+        <v>-26.64229202270508</v>
+      </c>
+      <c r="D1846">
+        <v>-31.61293411254883</v>
+      </c>
+      <c r="E1846">
+        <v>-29.40289115905762</v>
+      </c>
+    </row>
+    <row r="1847" spans="1:5">
+      <c r="A1847" s="1" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C1847">
+        <v>-23.46528625488281</v>
+      </c>
+      <c r="D1847">
+        <v>-19.79804611206055</v>
+      </c>
+      <c r="E1847">
+        <v>-18.66863250732422</v>
+      </c>
+    </row>
+    <row r="1848" spans="1:5">
+      <c r="A1848" s="1" t="s">
+        <v>1850</v>
+      </c>
+      <c r="C1848">
+        <v>138.2331390380859</v>
+      </c>
+      <c r="D1848">
+        <v>162.4386138916016</v>
+      </c>
+      <c r="E1848">
+        <v>170.8627471923828</v>
+      </c>
+    </row>
+    <row r="1849" spans="1:5">
+      <c r="A1849" s="1" t="s">
+        <v>1851</v>
+      </c>
+      <c r="C1849">
+        <v>-10.17635631561279</v>
+      </c>
+      <c r="D1849">
+        <v>-10.70745944976807</v>
+      </c>
+      <c r="E1849">
+        <v>-9.646365165710449</v>
+      </c>
+    </row>
+    <row r="1850" spans="1:5">
+      <c r="A1850" s="1" t="s">
+        <v>1852</v>
+      </c>
+      <c r="C1850">
+        <v>43.4904670715332</v>
+      </c>
+      <c r="D1850">
+        <v>-100</v>
+      </c>
+      <c r="E1850">
+        <v>53.30073547363281</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:5">
+      <c r="A1851" s="1" t="s">
+        <v>1853</v>
+      </c>
+      <c r="C1851">
+        <v>-22.16069221496582</v>
+      </c>
+      <c r="D1851">
+        <v>-21.57657432556152</v>
+      </c>
+      <c r="E1851">
+        <v>-19.96999931335449</v>
+      </c>
+    </row>
+    <row r="1852" spans="1:5">
+      <c r="A1852" s="1" t="s">
+        <v>1854</v>
+      </c>
+      <c r="C1852">
+        <v>-23.71253204345703</v>
+      </c>
+      <c r="D1852">
+        <v>-25.97347068786621</v>
+      </c>
+      <c r="E1852">
+        <v>-25.61108779907227</v>
+      </c>
+    </row>
+    <row r="1853" spans="1:5">
+      <c r="A1853" s="1" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C1853">
+        <v>-30.15028762817383</v>
+      </c>
+      <c r="D1853">
+        <v>-33.98865127563477</v>
+      </c>
+      <c r="E1853">
+        <v>-32.14559173583984</v>
+      </c>
+    </row>
+    <row r="1854" spans="1:5">
+      <c r="A1854" s="1" t="s">
+        <v>1856</v>
+      </c>
+      <c r="C1854">
+        <v>-100</v>
+      </c>
+      <c r="D1854">
+        <v>-100</v>
+      </c>
+      <c r="E1854">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1855" spans="1:5">
+      <c r="A1855" s="1" t="s">
+        <v>1857</v>
+      </c>
+      <c r="C1855">
+        <v>-29.41009140014648</v>
+      </c>
+      <c r="D1855">
+        <v>-29.41009140014648</v>
+      </c>
+      <c r="E1855">
+        <v>-29.41009140014648</v>
+      </c>
+    </row>
+    <row r="1856" spans="1:5">
+      <c r="A1856" s="1" t="s">
+        <v>1858</v>
+      </c>
+      <c r="C1856">
+        <v>-25.99195861816406</v>
+      </c>
+      <c r="D1856">
+        <v>-22.63495254516602</v>
+      </c>
+      <c r="E1856">
+        <v>-20.26705169677734</v>
+      </c>
+    </row>
+    <row r="1857" spans="1:5">
+      <c r="A1857" s="1" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C1857">
+        <v>-29.07699394226074</v>
+      </c>
+      <c r="D1857">
+        <v>-29.23058891296387</v>
+      </c>
+      <c r="E1857">
+        <v>-28.31185913085938</v>
+      </c>
+    </row>
+    <row r="1858" spans="1:5">
+      <c r="A1858" s="1" t="s">
+        <v>1860</v>
+      </c>
+      <c r="C1858">
+        <v>17.64059066772461</v>
+      </c>
+      <c r="D1858">
+        <v>8.361394882202148</v>
+      </c>
+      <c r="E1858">
+        <v>12.10616874694824</v>
+      </c>
+    </row>
+    <row r="1859" spans="1:5">
+      <c r="A1859" s="1" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C1859">
+        <v>-39.1231689453125</v>
+      </c>
+      <c r="D1859">
+        <v>-37.74115371704102</v>
+      </c>
+      <c r="E1859">
+        <v>-37.02981948852539</v>
+      </c>
+    </row>
+    <row r="1860" spans="1:5">
+      <c r="A1860" s="1" t="s">
+        <v>1862</v>
+      </c>
+      <c r="C1860">
+        <v>-88.8736572265625</v>
+      </c>
+      <c r="D1860">
+        <v>-89.00368499755859</v>
+      </c>
+      <c r="E1860">
+        <v>-88.78150939941406</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:5">
+      <c r="A1861" s="1" t="s">
+        <v>1863</v>
+      </c>
+      <c r="C1861">
+        <v>249.8621673583984</v>
+      </c>
+      <c r="D1861">
+        <v>265.9898376464844</v>
+      </c>
+      <c r="E1861">
+        <v>277.5034484863281</v>
+      </c>
+    </row>
+    <row r="1862" spans="1:5">
+      <c r="A1862" s="1" t="s">
+        <v>1864</v>
+      </c>
+      <c r="C1862">
+        <v>-21.96667289733887</v>
+      </c>
+      <c r="D1862">
+        <v>-20.1750545501709</v>
+      </c>
+      <c r="E1862">
+        <v>-16.58968353271484</v>
+      </c>
+    </row>
+    <row r="1863" spans="1:5">
+      <c r="A1863" s="1" t="s">
+        <v>1865</v>
+      </c>
+      <c r="C1863">
+        <v>-99.01702880859375</v>
+      </c>
+      <c r="D1863">
+        <v>-99.02851867675781</v>
+      </c>
+      <c r="E1863">
+        <v>-99.00888824462891</v>
+      </c>
+    </row>
+    <row r="1864" spans="1:5">
+      <c r="A1864" s="1" t="s">
+        <v>1866</v>
+      </c>
+      <c r="C1864">
+        <v>-97.70296478271484</v>
+      </c>
+      <c r="D1864">
+        <v>-97.72980499267578</v>
+      </c>
+      <c r="E1864">
+        <v>-97.68393707275391</v>
+      </c>
+    </row>
+    <row r="1865" spans="1:5">
+      <c r="A1865" s="1" t="s">
+        <v>1867</v>
+      </c>
+      <c r="C1865">
+        <v>-85.38395690917969</v>
+      </c>
+      <c r="D1865">
+        <v>-85.55476379394531</v>
+      </c>
+      <c r="E1865">
+        <v>-85.26290130615234</v>
+      </c>
+    </row>
+    <row r="1866" spans="1:5">
+      <c r="A1866" s="1" t="s">
+        <v>1868</v>
+      </c>
+      <c r="C1866">
+        <v>-94.00336456298828</v>
+      </c>
+      <c r="D1866">
+        <v>-94.07344818115234</v>
+      </c>
+      <c r="E1866">
+        <v>-93.95370483398438</v>
+      </c>
+    </row>
+    <row r="1867" spans="1:5">
+      <c r="A1867" s="1" t="s">
+        <v>1869</v>
+      </c>
+      <c r="C1867">
+        <v>-27.35002708435059</v>
+      </c>
+      <c r="D1867">
+        <v>-27.77956199645996</v>
+      </c>
+      <c r="E1867">
+        <v>-26.5982551574707</v>
+      </c>
+    </row>
+    <row r="1868" spans="1:5">
+      <c r="A1868" s="1" t="s">
+        <v>1870</v>
+      </c>
+      <c r="C1868">
+        <v>6.862723827362061</v>
+      </c>
+      <c r="D1868">
+        <v>-100</v>
+      </c>
+      <c r="E1868">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1869" spans="1:5">
+      <c r="A1869" s="1" t="s">
+        <v>1871</v>
+      </c>
+      <c r="C1869">
+        <v>7.58171272277832</v>
+      </c>
+    </row>
+    <row r="1870" spans="1:5">
+      <c r="A1870" s="1" t="s">
+        <v>1872</v>
+      </c>
+      <c r="C1870">
+        <v>24.05439949035645</v>
+      </c>
+      <c r="D1870">
+        <v>10.6007251739502</v>
+      </c>
+      <c r="E1870">
+        <v>13.46783351898193</v>
+      </c>
+    </row>
+    <row r="1871" spans="1:5">
+      <c r="A1871" s="1" t="s">
+        <v>1873</v>
+      </c>
+      <c r="C1871">
+        <v>2657.453125</v>
+      </c>
+      <c r="D1871">
+        <v>12.02837181091309</v>
+      </c>
+      <c r="E1871">
+        <v>15.17903900146484</v>
+      </c>
+    </row>
+    <row r="1872" spans="1:5">
+      <c r="A1872" s="1" t="s">
+        <v>1874</v>
+      </c>
+      <c r="C1872">
+        <v>25.22663307189941</v>
+      </c>
+      <c r="D1872">
+        <v>25.99800300598145</v>
+      </c>
+      <c r="E1872">
+        <v>27.37622261047363</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:5">
+      <c r="A1873" s="1" t="s">
+        <v>1875</v>
+      </c>
+      <c r="C1873">
+        <v>903.446044921875</v>
+      </c>
+      <c r="D1873">
+        <v>780.440185546875</v>
+      </c>
+      <c r="E1873">
+        <v>796.982666015625</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:5">
+      <c r="A1874" s="1" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C1874">
+        <v>27.49294853210449</v>
+      </c>
+      <c r="D1874">
+        <v>-100</v>
+      </c>
+      <c r="E1874">
+        <v>16.58352088928223</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:5">
+      <c r="A1875" s="1" t="s">
+        <v>1877</v>
+      </c>
+      <c r="C1875">
+        <v>27.82895469665527</v>
+      </c>
+      <c r="D1875">
+        <v>28.59170532226562</v>
+      </c>
+      <c r="E1875">
+        <v>35.24016571044922</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:5">
+      <c r="A1876" s="1" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C1876">
+        <v>11.80511569976807</v>
+      </c>
+      <c r="D1876">
+        <v>9.253467559814453</v>
+      </c>
+      <c r="E1876">
+        <v>16.24175643920898</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:5">
+      <c r="A1877" s="1" t="s">
+        <v>1879</v>
+      </c>
+      <c r="C1877">
+        <v>18.82792282104492</v>
+      </c>
+      <c r="D1877">
+        <v>14.69610500335693</v>
+      </c>
+      <c r="E1877">
+        <v>22.01045989990234</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:5">
+      <c r="A1878" s="1" t="s">
+        <v>1880</v>
+      </c>
+      <c r="C1878">
+        <v>6.692920684814453</v>
+      </c>
+      <c r="D1878">
+        <v>3.490712404251099</v>
+      </c>
+      <c r="E1878">
+        <v>4.539451599121094</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:5">
+      <c r="A1879" s="1" t="s">
+        <v>1881</v>
+      </c>
+      <c r="C1879">
+        <v>1.643964290618896</v>
+      </c>
+      <c r="E1879">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:5">
+      <c r="A1880" s="1" t="s">
+        <v>1882</v>
+      </c>
+      <c r="C1880">
+        <v>22.28820610046387</v>
+      </c>
+      <c r="D1880">
+        <v>3.529137849807739</v>
+      </c>
+      <c r="E1880">
+        <v>7.26594352722168</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:5">
+      <c r="A1881" s="1" t="s">
+        <v>1883</v>
+      </c>
+      <c r="C1881">
+        <v>7.137650489807129</v>
+      </c>
+      <c r="D1881">
+        <v>4.957151889801025</v>
+      </c>
+      <c r="E1881">
+        <v>5.108507633209229</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:5">
+      <c r="A1882" s="1" t="s">
+        <v>1884</v>
+      </c>
+      <c r="C1882">
+        <v>20.13122367858887</v>
+      </c>
+      <c r="D1882">
+        <v>14.03321838378906</v>
+      </c>
+      <c r="E1882">
+        <v>17.37783241271973</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:5">
+      <c r="A1883" s="1" t="s">
+        <v>1885</v>
+      </c>
+      <c r="C1883" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:5">
+      <c r="A1884" s="1" t="s">
+        <v>1886</v>
+      </c>
+      <c r="C1884">
+        <v>17.09033584594727</v>
+      </c>
+      <c r="D1884">
+        <v>17.09033584594727</v>
+      </c>
+      <c r="E1884">
+        <v>17.09033584594727</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:5">
+      <c r="A1885" s="1" t="s">
+        <v>1887</v>
+      </c>
+      <c r="C1885">
+        <v>9.402849197387695</v>
+      </c>
+      <c r="D1885">
+        <v>6.647522926330566</v>
+      </c>
+      <c r="E1885">
+        <v>11.64308643341064</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:5">
+      <c r="A1886" s="1" t="s">
+        <v>1888</v>
+      </c>
+      <c r="C1886">
+        <v>15.52823543548584</v>
+      </c>
+      <c r="D1886">
+        <v>1.851727604866028</v>
+      </c>
+      <c r="E1886">
+        <v>6.139818668365479</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:5">
+      <c r="A1887" s="1" t="s">
+        <v>1889</v>
+      </c>
+      <c r="C1887">
+        <v>9.152072906494141</v>
+      </c>
+      <c r="D1887">
+        <v>3.019472599029541</v>
+      </c>
+      <c r="E1887">
+        <v>5.885316371917725</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:5">
+      <c r="A1888" s="1" t="s">
+        <v>1890</v>
+      </c>
+      <c r="C1888">
+        <v>17.12021064758301</v>
+      </c>
+      <c r="D1888">
+        <v>5.537042617797852</v>
+      </c>
+      <c r="E1888">
+        <v>7.69061279296875</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:5">
+      <c r="A1889" s="1" t="s">
+        <v>1891</v>
+      </c>
+      <c r="C1889">
+        <v>1246.728271484375</v>
+      </c>
+      <c r="D1889">
+        <v>1134.054565429688</v>
+      </c>
+      <c r="E1889">
+        <v>1155.896606445312</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:5">
+      <c r="A1890" s="1" t="s">
+        <v>1892</v>
+      </c>
+      <c r="C1890">
+        <v>32.31802749633789</v>
+      </c>
+      <c r="D1890">
+        <v>29.08674812316895</v>
+      </c>
+      <c r="E1890">
+        <v>35.35954666137695</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:5">
+      <c r="A1891" s="1" t="s">
+        <v>1893</v>
+      </c>
+      <c r="C1891">
+        <v>16.34242248535156</v>
+      </c>
+      <c r="D1891">
+        <v>3.881914377212524</v>
+      </c>
+      <c r="E1891">
+        <v>7.013106346130371</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:5">
+      <c r="A1892" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C1892">
+        <v>7679.8896484375</v>
+      </c>
+      <c r="D1892">
+        <v>6154.1376953125</v>
+      </c>
+      <c r="E1892">
+        <v>6765.2626953125</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:5">
+      <c r="A1893" s="1" t="s">
+        <v>1895</v>
+      </c>
+      <c r="C1893">
+        <v>2312.51416015625</v>
+      </c>
+      <c r="D1893">
+        <v>12.02837181091309</v>
+      </c>
+      <c r="E1893">
+        <v>15.17903900146484</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:5">
+      <c r="A1894" s="1" t="s">
+        <v>1896</v>
+      </c>
+      <c r="C1894">
+        <v>667.0103149414062</v>
+      </c>
+      <c r="D1894">
+        <v>641.07568359375</v>
+      </c>
+      <c r="E1894">
+        <v>605.4154052734375</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:5">
+      <c r="A1895" s="1" t="s">
+        <v>1897</v>
+      </c>
+      <c r="C1895">
+        <v>753.2020263671875</v>
+      </c>
+      <c r="D1895">
+        <v>12.02837181091309</v>
+      </c>
+      <c r="E1895">
+        <v>15.17903900146484</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:5">
+      <c r="A1896" s="1" t="s">
+        <v>1898</v>
+      </c>
+      <c r="C1896">
+        <v>11.64621639251709</v>
+      </c>
+      <c r="D1896">
+        <v>-94.14774322509766</v>
+      </c>
+      <c r="E1896">
+        <v>2.993500709533691</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:5">
+      <c r="A1897" s="1" t="s">
+        <v>1899</v>
+      </c>
+      <c r="C1897">
+        <v>7.468527317047119</v>
+      </c>
+      <c r="D1897" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1897" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:5">
+      <c r="A1898" s="1" t="s">
+        <v>1900</v>
+      </c>
+      <c r="C1898">
+        <v>8.318314552307129</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:5">
+      <c r="A1899" s="1" t="s">
+        <v>1901</v>
+      </c>
+      <c r="C1899">
+        <v>8.760002136230469</v>
+      </c>
+      <c r="D1899">
+        <v>-99.64057159423828</v>
+      </c>
+      <c r="E1899">
+        <v>-99.62746429443359</v>
+      </c>
+    </row>
+    <row r="1900" spans="1:5">
+      <c r="A1900" s="1" t="s">
+        <v>1902</v>
+      </c>
+      <c r="C1900">
+        <v>13.06198024749756</v>
+      </c>
+      <c r="D1900">
+        <v>2262.28076171875</v>
+      </c>
+      <c r="E1900">
+        <v>2295.578369140625</v>
+      </c>
+    </row>
+    <row r="1901" spans="1:5">
+      <c r="A1901" s="1" t="s">
+        <v>1903</v>
+      </c>
+      <c r="C1901">
+        <v>3.836580038070679</v>
+      </c>
+      <c r="D1901">
+        <v>17.32173728942871</v>
+      </c>
+      <c r="E1901">
+        <v>20.05820655822754</v>
+      </c>
+    </row>
+    <row r="1902" spans="1:5">
+      <c r="A1902" s="1" t="s">
+        <v>1904</v>
+      </c>
+      <c r="C1902">
+        <v>4.046356201171875</v>
+      </c>
+      <c r="D1902">
+        <v>-85.02593994140625</v>
+      </c>
+      <c r="E1902">
+        <v>-84.51177978515625</v>
+      </c>
+    </row>
+    <row r="1903" spans="1:5">
+      <c r="A1903" s="1" t="s">
+        <v>1905</v>
+      </c>
+      <c r="C1903">
+        <v>22.17300224304199</v>
+      </c>
+      <c r="D1903" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1903">
+        <v>15.68651962280273</v>
+      </c>
+    </row>
+    <row r="1904" spans="1:5">
+      <c r="A1904" s="1" t="s">
+        <v>1906</v>
+      </c>
+      <c r="C1904">
+        <v>20.58630561828613</v>
+      </c>
+      <c r="D1904">
+        <v>19.47366905212402</v>
+      </c>
+      <c r="E1904">
+        <v>22.5789794921875</v>
+      </c>
+    </row>
+    <row r="1905" spans="1:5">
+      <c r="A1905" s="1" t="s">
+        <v>1907</v>
+      </c>
+      <c r="C1905">
+        <v>12.10302829742432</v>
+      </c>
+      <c r="D1905">
+        <v>9.294498443603516</v>
+      </c>
+      <c r="E1905">
+        <v>13.84101581573486</v>
+      </c>
+    </row>
+    <row r="1906" spans="1:5">
+      <c r="A1906" s="1" t="s">
+        <v>1908</v>
+      </c>
+      <c r="C1906">
+        <v>7.851326465606689</v>
+      </c>
+      <c r="D1906">
+        <v>-69.68054962158203</v>
+      </c>
+      <c r="E1906">
+        <v>-68.89122009277344</v>
+      </c>
+    </row>
+    <row r="1907" spans="1:5">
+      <c r="A1907" s="1" t="s">
+        <v>1909</v>
+      </c>
+      <c r="C1907">
+        <v>7.136096477508545</v>
+      </c>
+      <c r="D1907">
+        <v>5.08370304107666</v>
+      </c>
+      <c r="E1907">
+        <v>6.099717140197754</v>
+      </c>
+    </row>
+    <row r="1908" spans="1:5">
+      <c r="A1908" s="1" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C1908">
+        <v>0.4043438136577606</v>
+      </c>
+    </row>
+    <row r="1909" spans="1:5">
+      <c r="A1909" s="1" t="s">
+        <v>1911</v>
+      </c>
+      <c r="C1909">
+        <v>18.1339111328125</v>
+      </c>
+      <c r="D1909">
+        <v>3.263134002685547</v>
+      </c>
+      <c r="E1909">
+        <v>14.61375045776367</v>
+      </c>
+    </row>
+    <row r="1910" spans="1:5">
+      <c r="A1910" s="1" t="s">
+        <v>1912</v>
+      </c>
+      <c r="C1910">
+        <v>8.71646785736084</v>
+      </c>
+      <c r="D1910">
+        <v>4.783885478973389</v>
+      </c>
+      <c r="E1910">
+        <v>6.025421619415283</v>
+      </c>
+    </row>
+    <row r="1911" spans="1:5">
+      <c r="A1911" s="1" t="s">
+        <v>1913</v>
+      </c>
+      <c r="C1911">
+        <v>7.151594161987305</v>
+      </c>
+      <c r="D1911">
+        <v>2.854996204376221</v>
+      </c>
+      <c r="E1911">
+        <v>4.24039888381958</v>
+      </c>
+    </row>
+    <row r="1912" spans="1:5">
+      <c r="A1912" s="1" t="s">
+        <v>1914</v>
+      </c>
+      <c r="C1912">
+        <v>6.514657974243164</v>
+      </c>
+    </row>
+    <row r="1913" spans="1:5">
+      <c r="A1913" s="1" t="s">
+        <v>1915</v>
+      </c>
+      <c r="C1913">
+        <v>22.69301605224609</v>
+      </c>
+      <c r="D1913">
+        <v>22.69301605224609</v>
+      </c>
+      <c r="E1913">
+        <v>22.69301605224609</v>
+      </c>
+    </row>
+    <row r="1914" spans="1:5">
+      <c r="A1914" s="1" t="s">
+        <v>1916</v>
+      </c>
+      <c r="C1914">
+        <v>5.309175491333008</v>
+      </c>
+      <c r="D1914">
+        <v>3.499712944030762</v>
+      </c>
+      <c r="E1914">
+        <v>7.045456886291504</v>
+      </c>
+    </row>
+    <row r="1915" spans="1:5">
+      <c r="A1915" s="1" t="s">
+        <v>1917</v>
+      </c>
+      <c r="C1915">
+        <v>16.73989486694336</v>
+      </c>
+      <c r="D1915">
+        <v>6.554084300994873</v>
+      </c>
+      <c r="E1915">
+        <v>14.0118465423584</v>
+      </c>
+    </row>
+    <row r="1916" spans="1:5">
+      <c r="A1916" s="1" t="s">
+        <v>1918</v>
+      </c>
+      <c r="C1916">
+        <v>43.83361434936523</v>
+      </c>
+      <c r="D1916">
+        <v>33.55083847045898</v>
+      </c>
+      <c r="E1916">
+        <v>32.8935661315918</v>
+      </c>
+    </row>
+    <row r="1917" spans="1:5">
+      <c r="A1917" s="1" t="s">
+        <v>1919</v>
+      </c>
+      <c r="C1917">
+        <v>13.81486988067627</v>
+      </c>
+      <c r="D1917">
+        <v>20.50991439819336</v>
+      </c>
+      <c r="E1917">
+        <v>31.8197078704834</v>
+      </c>
+    </row>
+    <row r="1918" spans="1:5">
+      <c r="A1918" s="1" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C1918">
+        <v>7.464813232421875</v>
+      </c>
+      <c r="D1918">
+        <v>-89.31671142578125</v>
+      </c>
+      <c r="E1918">
+        <v>-88.93804931640625</v>
+      </c>
+    </row>
+    <row r="1919" spans="1:5">
+      <c r="A1919" s="1" t="s">
+        <v>1921</v>
+      </c>
+      <c r="C1919">
+        <v>15.54188823699951</v>
+      </c>
+      <c r="D1919">
+        <v>12.45337200164795</v>
+      </c>
+      <c r="E1919">
+        <v>17.29500770568848</v>
+      </c>
+    </row>
+    <row r="1920" spans="1:5">
+      <c r="A1920" s="1" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C1920">
+        <v>12.48497772216797</v>
+      </c>
+      <c r="D1920">
+        <v>-96.79002380371094</v>
+      </c>
+      <c r="E1920">
+        <v>2.522807598114014</v>
+      </c>
+    </row>
+    <row r="1921" spans="1:5">
+      <c r="A1921" s="1" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C1921">
+        <v>42.09703063964844</v>
+      </c>
+      <c r="D1921">
+        <v>22.67024040222168</v>
+      </c>
+      <c r="E1921">
+        <v>36.33816909790039</v>
+      </c>
+    </row>
+    <row r="1922" spans="1:5">
+      <c r="A1922" s="1" t="s">
+        <v>1924</v>
+      </c>
+      <c r="C1922">
+        <v>11.00553321838379</v>
+      </c>
+      <c r="D1922">
+        <v>17.68236923217773</v>
+      </c>
+      <c r="E1922">
+        <v>20.61801719665527</v>
+      </c>
+    </row>
+    <row r="1923" spans="1:5">
+      <c r="A1923" s="1" t="s">
+        <v>1925</v>
+      </c>
+      <c r="C1923">
+        <v>9.618955612182617</v>
+      </c>
+      <c r="D1923">
+        <v>11.66934490203857</v>
+      </c>
+      <c r="E1923">
+        <v>11.94405364990234</v>
+      </c>
+    </row>
+    <row r="1924" spans="1:5">
+      <c r="A1924" s="1" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1924">
+        <v>7.006062030792236</v>
+      </c>
+      <c r="D1924">
+        <v>17.68236923217773</v>
+      </c>
+      <c r="E1924">
+        <v>20.61801719665527</v>
+      </c>
+    </row>
+    <row r="1925" spans="1:5">
+      <c r="A1925" s="1" t="s">
+        <v>1927</v>
+      </c>
+      <c r="C1925">
+        <v>9.17125415802002</v>
+      </c>
+      <c r="D1925">
+        <v>1625.178588867188</v>
+      </c>
+      <c r="E1925">
+        <v>2.40341854095459</v>
+      </c>
+    </row>
+    <row r="1926" spans="1:5">
+      <c r="A1926" s="1" t="s">
+        <v>1928</v>
+      </c>
+      <c r="C1926">
+        <v>8.000015258789062</v>
+      </c>
+      <c r="D1926">
+        <v>3.901735305786133</v>
+      </c>
+      <c r="E1926">
+        <v>5.82514762878418</v>
+      </c>
+    </row>
+    <row r="1927" spans="1:5">
+      <c r="A1927" s="1" t="s">
+        <v>1929</v>
+      </c>
+      <c r="C1927">
+        <v>18.00707054138184</v>
+      </c>
+      <c r="D1927" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1927" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1928" spans="1:5">
+      <c r="A1928" s="1" t="s">
+        <v>1930</v>
+      </c>
+      <c r="C1928">
+        <v>8.043951034545898</v>
+      </c>
+      <c r="D1928">
+        <v>29602.5546875</v>
+      </c>
+      <c r="E1928">
+        <v>28343.052734375</v>
+      </c>
+    </row>
+    <row r="1929" spans="1:5">
+      <c r="A1929" s="1" t="s">
+        <v>1931</v>
+      </c>
+      <c r="C1929">
+        <v>11.10453128814697</v>
+      </c>
+      <c r="D1929">
+        <v>13.94086265563965</v>
+      </c>
+      <c r="E1929">
+        <v>25.02372550964355</v>
+      </c>
+    </row>
+    <row r="1930" spans="1:5">
+      <c r="A1930" s="1" t="s">
+        <v>1932</v>
+      </c>
+      <c r="C1930">
+        <v>2.330730676651001</v>
+      </c>
+      <c r="D1930">
+        <v>11.10030174255371</v>
+      </c>
+      <c r="E1930">
+        <v>12.53560543060303</v>
+      </c>
+    </row>
+    <row r="1931" spans="1:5">
+      <c r="A1931" s="1" t="s">
+        <v>1933</v>
+      </c>
+      <c r="C1931">
+        <v>3.449650526046753</v>
+      </c>
+      <c r="D1931">
+        <v>582.2554321289062</v>
+      </c>
+      <c r="E1931">
+        <v>21.28029632568359</v>
+      </c>
+    </row>
+    <row r="1932" spans="1:5">
+      <c r="A1932" s="1" t="s">
+        <v>1934</v>
+      </c>
+      <c r="C1932">
+        <v>17.85250663757324</v>
+      </c>
+      <c r="D1932">
+        <v>11.73312568664551</v>
+      </c>
+      <c r="E1932">
+        <v>12.11813449859619</v>
+      </c>
+    </row>
+    <row r="1933" spans="1:5">
+      <c r="A1933" s="1" t="s">
+        <v>1935</v>
+      </c>
+      <c r="C1933">
+        <v>10.27401828765869</v>
+      </c>
+      <c r="D1933">
+        <v>4.47040319442749</v>
+      </c>
+      <c r="E1933">
+        <v>7.517856597900391</v>
+      </c>
+    </row>
+    <row r="1934" spans="1:5">
+      <c r="A1934" s="1" t="s">
+        <v>1936</v>
+      </c>
+      <c r="C1934">
+        <v>11.84947204589844</v>
+      </c>
+      <c r="D1934">
+        <v>6.557873725891113</v>
+      </c>
+      <c r="E1934">
+        <v>8.900356292724609</v>
+      </c>
+    </row>
+    <row r="1935" spans="1:5">
+      <c r="A1935" s="1" t="s">
+        <v>1937</v>
+      </c>
+      <c r="C1935">
+        <v>15.08343124389648</v>
+      </c>
+      <c r="D1935">
+        <v>260.1383056640625</v>
+      </c>
+      <c r="E1935">
+        <v>283.6507568359375</v>
+      </c>
+    </row>
+    <row r="1936" spans="1:5">
+      <c r="A1936" s="1" t="s">
+        <v>1938</v>
+      </c>
+      <c r="C1936">
+        <v>20.92133712768555</v>
+      </c>
+      <c r="D1936">
+        <v>19.52780151367188</v>
+      </c>
+      <c r="E1936">
+        <v>45.95585632324219</v>
+      </c>
+    </row>
+    <row r="1937" spans="1:5">
+      <c r="A1937" s="1" t="s">
+        <v>1939</v>
+      </c>
+      <c r="C1937">
+        <v>0.4027154445648193</v>
+      </c>
+    </row>
+    <row r="1938" spans="1:5">
+      <c r="A1938" s="1" t="s">
+        <v>1940</v>
+      </c>
+      <c r="C1938">
+        <v>14.06790542602539</v>
+      </c>
+      <c r="D1938">
+        <v>9.393896102905273</v>
+      </c>
+      <c r="E1938">
+        <v>10.7661018371582</v>
+      </c>
+    </row>
+    <row r="1939" spans="1:5">
+      <c r="A1939" s="1" t="s">
+        <v>1941</v>
+      </c>
+      <c r="C1939">
+        <v>7.772922515869141</v>
+      </c>
+      <c r="D1939">
+        <v>5.264143466949463</v>
+      </c>
+      <c r="E1939">
+        <v>8.392663955688477</v>
+      </c>
+    </row>
+    <row r="1940" spans="1:5">
+      <c r="A1940" s="1" t="s">
+        <v>1942</v>
+      </c>
+      <c r="C1940">
+        <v>17.69796943664551</v>
+      </c>
+      <c r="D1940">
+        <v>1.137654304504395</v>
+      </c>
+      <c r="E1940">
+        <v>3.189161539077759</v>
+      </c>
+    </row>
+    <row r="1941" spans="1:5">
+      <c r="A1941" s="1" t="s">
+        <v>1943</v>
+      </c>
+      <c r="C1941">
+        <v>6.116208076477051</v>
+      </c>
+      <c r="D1941" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1942" spans="1:5">
+      <c r="A1942" s="1" t="s">
+        <v>1944</v>
+      </c>
+      <c r="C1942">
+        <v>15.85595703125</v>
+      </c>
+      <c r="D1942">
+        <v>15.85595703125</v>
+      </c>
+      <c r="E1942">
+        <v>15.85595703125</v>
+      </c>
+    </row>
+    <row r="1943" spans="1:5">
+      <c r="A1943" s="1" t="s">
+        <v>1945</v>
+      </c>
+      <c r="C1943">
+        <v>4.366089820861816</v>
+      </c>
+      <c r="D1943">
+        <v>1.675084471702576</v>
+      </c>
+      <c r="E1943">
+        <v>3.053096055984497</v>
+      </c>
+    </row>
+    <row r="1944" spans="1:5">
+      <c r="A1944" s="1" t="s">
+        <v>1946</v>
+      </c>
+      <c r="C1944">
+        <v>21.99891471862793</v>
+      </c>
+      <c r="D1944">
+        <v>7.843052387237549</v>
+      </c>
+      <c r="E1944">
+        <v>18.04816818237305</v>
+      </c>
+    </row>
+    <row r="1945" spans="1:5">
+      <c r="A1945" s="1" t="s">
+        <v>1947</v>
+      </c>
+      <c r="C1945">
+        <v>29.99481391906738</v>
+      </c>
+      <c r="D1945">
+        <v>25.09633636474609</v>
+      </c>
+      <c r="E1945">
+        <v>26.42307090759277</v>
+      </c>
+    </row>
+    <row r="1946" spans="1:5">
+      <c r="A1946" s="1" t="s">
+        <v>1948</v>
+      </c>
+      <c r="C1946">
+        <v>29.35686111450195</v>
+      </c>
+      <c r="D1946">
+        <v>59.33816146850586</v>
+      </c>
+      <c r="E1946">
+        <v>70.34635925292969</v>
+      </c>
+    </row>
+    <row r="1947" spans="1:5">
+      <c r="A1947" s="1" t="s">
+        <v>1949</v>
+      </c>
+      <c r="C1947">
+        <v>1.436096549034119</v>
+      </c>
+      <c r="D1947">
+        <v>16.96403312683105</v>
+      </c>
+      <c r="E1947">
+        <v>21.28029632568359</v>
+      </c>
+    </row>
+    <row r="1948" spans="1:5">
+      <c r="A1948" s="1" t="s">
+        <v>1950</v>
+      </c>
+      <c r="C1948">
+        <v>11.4394702911377</v>
+      </c>
+      <c r="D1948">
+        <v>5.691106796264648</v>
+      </c>
+      <c r="E1948">
+        <v>7.954504013061523</v>
+      </c>
+    </row>
+    <row r="1949" spans="1:5">
+      <c r="A1949" s="1" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C1949">
+        <v>11.00747966766357</v>
+      </c>
+      <c r="D1949">
+        <v>3064.06201171875</v>
+      </c>
+      <c r="E1949">
+        <v>5.331850051879883</v>
+      </c>
+    </row>
+    <row r="1950" spans="1:5">
+      <c r="A1950" s="1" t="s">
+        <v>1952</v>
+      </c>
+      <c r="C1950">
+        <v>18.76491355895996</v>
+      </c>
+      <c r="D1950">
+        <v>12.48562145233154</v>
+      </c>
+      <c r="E1950">
+        <v>13.15376281738281</v>
+      </c>
+    </row>
+    <row r="1951" spans="1:5">
+      <c r="A1951" s="1" t="s">
+        <v>1953</v>
+      </c>
+      <c r="C1951">
+        <v>9.910930633544922</v>
+      </c>
+      <c r="D1951">
+        <v>1630.290283203125</v>
+      </c>
+      <c r="E1951">
+        <v>1701.338256835938</v>
+      </c>
+    </row>
+    <row r="1952" spans="1:5">
+      <c r="A1952" s="1" t="s">
+        <v>1954</v>
+      </c>
+      <c r="C1952">
+        <v>8.229348182678223</v>
+      </c>
+      <c r="D1952">
+        <v>5.859855651855469</v>
+      </c>
+      <c r="E1952">
+        <v>7.219461917877197</v>
+      </c>
+    </row>
+    <row r="1953" spans="1:5">
+      <c r="A1953" s="1" t="s">
+        <v>1955</v>
+      </c>
+      <c r="C1953">
+        <v>70.09065246582031</v>
+      </c>
+      <c r="D1953">
+        <v>817.7852783203125</v>
+      </c>
+      <c r="E1953">
+        <v>867.1316528320312</v>
+      </c>
+    </row>
+    <row r="1954" spans="1:5">
+      <c r="A1954" s="1" t="s">
+        <v>1956</v>
+      </c>
+      <c r="C1954">
+        <v>11.60948181152344</v>
+      </c>
+      <c r="D1954">
+        <v>1.506057262420654</v>
+      </c>
+      <c r="E1954">
+        <v>6.103707790374756</v>
+      </c>
+    </row>
+    <row r="1955" spans="1:5">
+      <c r="A1955" s="1" t="s">
+        <v>1957</v>
+      </c>
+      <c r="C1955">
+        <v>-100</v>
+      </c>
+      <c r="D1955">
+        <v>-100</v>
+      </c>
+      <c r="E1955">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1956" spans="1:5">
+      <c r="A1956" s="1" t="s">
+        <v>1958</v>
+      </c>
+      <c r="C1956">
+        <v>-100</v>
+      </c>
+      <c r="D1956">
+        <v>-100</v>
+      </c>
+      <c r="E1956">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1957" spans="1:5">
+      <c r="A1957" s="1" t="s">
+        <v>1959</v>
+      </c>
+      <c r="C1957">
+        <v>0.3800555467605591</v>
+      </c>
+      <c r="D1957">
+        <v>17.14908790588379</v>
+      </c>
+      <c r="E1957">
+        <v>9.923203468322754</v>
+      </c>
+    </row>
+    <row r="1958" spans="1:5">
+      <c r="A1958" s="1" t="s">
+        <v>1960</v>
+      </c>
+      <c r="C1958">
+        <v>0.7732897996902466</v>
+      </c>
+      <c r="D1958">
+        <v>3.639347791671753</v>
+      </c>
+      <c r="E1958">
+        <v>39.60202789306641</v>
+      </c>
+    </row>
+    <row r="1959" spans="1:5">
+      <c r="A1959" s="1" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C1959">
+        <v>2.592678546905518</v>
+      </c>
+      <c r="D1959">
+        <v>22.79574012756348</v>
+      </c>
+      <c r="E1959">
+        <v>24.56206703186035</v>
+      </c>
+    </row>
+    <row r="1960" spans="1:5">
+      <c r="A1960" s="1" t="s">
+        <v>1962</v>
+      </c>
+      <c r="C1960">
+        <v>4.663471698760986</v>
+      </c>
+      <c r="D1960">
+        <v>20.24318695068359</v>
+      </c>
+      <c r="E1960">
+        <v>522.3865356445312</v>
+      </c>
+    </row>
+    <row r="1961" spans="1:5">
+      <c r="A1961" s="1" t="s">
+        <v>1963</v>
+      </c>
+      <c r="C1961">
+        <v>24.07377815246582</v>
+      </c>
+      <c r="D1961">
+        <v>39.88592529296875</v>
+      </c>
+      <c r="E1961">
+        <v>35.90115737915039</v>
+      </c>
+    </row>
+    <row r="1962" spans="1:5">
+      <c r="A1962" s="1" t="s">
+        <v>1964</v>
+      </c>
+      <c r="C1962">
+        <v>3.406226396560669</v>
+      </c>
+      <c r="D1962">
+        <v>1.574849605560303</v>
+      </c>
+      <c r="E1962">
+        <v>3.970083236694336</v>
+      </c>
+    </row>
+    <row r="1963" spans="1:5">
+      <c r="A1963" s="1" t="s">
+        <v>1965</v>
+      </c>
+      <c r="C1963">
+        <v>1.955814480781555</v>
+      </c>
+      <c r="D1963">
+        <v>2.318260431289673</v>
+      </c>
+      <c r="E1963">
+        <v>3.032900333404541</v>
+      </c>
+    </row>
+    <row r="1964" spans="1:5">
+      <c r="A1964" s="1" t="s">
+        <v>1966</v>
+      </c>
+      <c r="C1964">
+        <v>9.736428260803223</v>
+      </c>
+      <c r="D1964">
+        <v>21.3304615020752</v>
+      </c>
+      <c r="E1964">
+        <v>22.41931343078613</v>
+      </c>
+    </row>
+    <row r="1965" spans="1:5">
+      <c r="A1965" s="1" t="s">
+        <v>1967</v>
+      </c>
+      <c r="C1965">
+        <v>9.909064292907715</v>
+      </c>
+      <c r="D1965">
+        <v>19.69295883178711</v>
+      </c>
+      <c r="E1965">
+        <v>39.79788970947266</v>
+      </c>
+    </row>
+    <row r="1966" spans="1:5">
+      <c r="A1966" s="1" t="s">
+        <v>1968</v>
+      </c>
+      <c r="C1966">
+        <v>0.4011001586914062</v>
+      </c>
+      <c r="D1966" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1966" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1967" spans="1:5">
+      <c r="A1967" s="1" t="s">
+        <v>1969</v>
+      </c>
+      <c r="C1967">
+        <v>7.203895568847656</v>
+      </c>
+      <c r="D1967">
+        <v>22.62425994873047</v>
+      </c>
+      <c r="E1967">
+        <v>17.17148017883301</v>
+      </c>
+    </row>
+    <row r="1968" spans="1:5">
+      <c r="A1968" s="1" t="s">
+        <v>1970</v>
+      </c>
+      <c r="C1968">
+        <v>7.024309635162354</v>
+      </c>
+      <c r="D1968">
+        <v>8.091565132141113</v>
+      </c>
+      <c r="E1968">
+        <v>11.07551765441895</v>
+      </c>
+    </row>
+    <row r="1969" spans="1:5">
+      <c r="A1969" s="1" t="s">
+        <v>1971</v>
+      </c>
+      <c r="C1969">
+        <v>4.059111595153809</v>
+      </c>
+      <c r="D1969">
+        <v>7.404355049133301</v>
+      </c>
+      <c r="E1969">
+        <v>9.057644844055176</v>
+      </c>
+    </row>
+    <row r="1970" spans="1:5">
+      <c r="A1970" s="1" t="s">
+        <v>1972</v>
+      </c>
+      <c r="C1970">
+        <v>-100</v>
+      </c>
+      <c r="D1970">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1971" spans="1:5">
+      <c r="A1971" s="1" t="s">
+        <v>1973</v>
+      </c>
+      <c r="C1971">
+        <v>0</v>
+      </c>
+      <c r="D1971">
+        <v>0</v>
+      </c>
+      <c r="E1971">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1972" spans="1:5">
+      <c r="A1972" s="1" t="s">
+        <v>1974</v>
+      </c>
+      <c r="C1972">
+        <v>2.626588106155396</v>
+      </c>
+      <c r="D1972">
+        <v>2.276456356048584</v>
+      </c>
+      <c r="E1972">
+        <v>3.594907522201538</v>
+      </c>
+    </row>
+    <row r="1973" spans="1:5">
+      <c r="A1973" s="1" t="s">
+        <v>1975</v>
+      </c>
+      <c r="C1973">
+        <v>9.776825904846191</v>
+      </c>
+      <c r="D1973">
+        <v>9.25357723236084</v>
+      </c>
+      <c r="E1973">
+        <v>20.41475105285645</v>
+      </c>
+    </row>
+    <row r="1974" spans="1:5">
+      <c r="A1974" s="1" t="s">
+        <v>1976</v>
+      </c>
+      <c r="C1974">
+        <v>-3.59332275390625</v>
+      </c>
+      <c r="D1974">
+        <v>-42.47799301147461</v>
+      </c>
+      <c r="E1974">
+        <v>4.293241024017334</v>
+      </c>
+    </row>
+    <row r="1975" spans="1:5">
+      <c r="A1975" s="1" t="s">
+        <v>1977</v>
+      </c>
+      <c r="C1975">
+        <v>11.90443992614746</v>
+      </c>
+      <c r="D1975">
+        <v>41.63571166992188</v>
+      </c>
+      <c r="E1975">
+        <v>46.91225433349609</v>
+      </c>
+    </row>
+    <row r="1976" spans="1:5">
+      <c r="A1976" s="1" t="s">
+        <v>1978</v>
+      </c>
+      <c r="C1976">
+        <v>2.393425941467285</v>
+      </c>
+      <c r="D1976">
+        <v>848.453125</v>
+      </c>
+      <c r="E1976">
+        <v>740.5821533203125</v>
+      </c>
+    </row>
+    <row r="1977" spans="1:5">
+      <c r="A1977" s="1" t="s">
+        <v>1979</v>
+      </c>
+      <c r="C1977">
+        <v>3.402884721755981</v>
+      </c>
+      <c r="D1977">
+        <v>10.24697780609131</v>
+      </c>
+      <c r="E1977">
+        <v>11.45570468902588</v>
+      </c>
+    </row>
+    <row r="1978" spans="1:5">
+      <c r="A1978" s="1" t="s">
+        <v>1980</v>
+      </c>
+      <c r="C1978">
+        <v>2.553990125656128</v>
+      </c>
+      <c r="D1978">
+        <v>6.50149393081665</v>
+      </c>
+      <c r="E1978">
+        <v>6.499076843261719</v>
+      </c>
+    </row>
+    <row r="1979" spans="1:5">
+      <c r="A1979" s="1" t="s">
+        <v>1981</v>
+      </c>
+      <c r="C1979">
+        <v>13.32607173919678</v>
+      </c>
+      <c r="D1979">
+        <v>30.6917610168457</v>
+      </c>
+      <c r="E1979">
+        <v>24.96785736083984</v>
+      </c>
+    </row>
+    <row r="1980" spans="1:5">
+      <c r="A1980" s="1" t="s">
+        <v>1982</v>
+      </c>
+      <c r="C1980">
+        <v>-94.15592956542969</v>
+      </c>
+      <c r="D1980">
+        <v>-92.28206634521484</v>
+      </c>
+      <c r="E1980">
+        <v>-92.04338073730469</v>
+      </c>
+    </row>
+    <row r="1981" spans="1:5">
+      <c r="A1981" s="1" t="s">
+        <v>1983</v>
+      </c>
+      <c r="C1981">
+        <v>-81.09664154052734</v>
+      </c>
+      <c r="D1981">
+        <v>-79.90297698974609</v>
+      </c>
+      <c r="E1981">
+        <v>-76.48257446289062</v>
+      </c>
+    </row>
+    <row r="1982" spans="1:5">
+      <c r="A1982" s="1" t="s">
+        <v>1984</v>
+      </c>
+      <c r="C1982">
+        <v>13.64478874206543</v>
+      </c>
+      <c r="D1982">
+        <v>26.05955505371094</v>
+      </c>
+      <c r="E1982">
+        <v>23.21361351013184</v>
+      </c>
+    </row>
+    <row r="1983" spans="1:5">
+      <c r="A1983" s="1" t="s">
+        <v>1985</v>
+      </c>
+      <c r="C1983">
+        <v>2.479773044586182</v>
+      </c>
+      <c r="D1983">
+        <v>5.608715534210205</v>
+      </c>
+      <c r="E1983">
+        <v>9.677143096923828</v>
+      </c>
+    </row>
+    <row r="1984" spans="1:5">
+      <c r="A1984" s="1" t="s">
+        <v>1986</v>
+      </c>
+      <c r="C1984" t="s">
+        <v>2024</v>
+      </c>
+      <c r="D1984" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1984" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1985" spans="1:5">
+      <c r="A1985" s="1" t="s">
+        <v>1987</v>
+      </c>
+      <c r="C1985" t="s">
+        <v>2024</v>
+      </c>
+      <c r="D1985" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1985" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1986" spans="1:5">
+      <c r="A1986" s="1" t="s">
+        <v>1988</v>
+      </c>
+      <c r="C1986">
+        <v>0.3451904952526093</v>
+      </c>
+      <c r="D1986">
+        <v>3.687396287918091</v>
+      </c>
+      <c r="E1986">
+        <v>-99.46699523925781</v>
+      </c>
+    </row>
+    <row r="1987" spans="1:5">
+      <c r="A1987" s="1" t="s">
+        <v>1989</v>
+      </c>
+      <c r="C1987">
+        <v>0.3129008412361145</v>
+      </c>
+      <c r="D1987">
+        <v>50.03044128417969</v>
+      </c>
+      <c r="E1987">
+        <v>72.09524536132812</v>
+      </c>
+    </row>
+    <row r="1988" spans="1:5">
+      <c r="A1988" s="1" t="s">
+        <v>1990</v>
+      </c>
+      <c r="C1988">
+        <v>2.811794519424438</v>
+      </c>
+      <c r="D1988">
+        <v>17.21816825866699</v>
+      </c>
+      <c r="E1988">
+        <v>18.66708755493164</v>
+      </c>
+    </row>
+    <row r="1989" spans="1:5">
+      <c r="A1989" s="1" t="s">
+        <v>1991</v>
+      </c>
+      <c r="C1989">
+        <v>3.052391052246094</v>
+      </c>
+      <c r="D1989">
+        <v>6.871538639068604</v>
+      </c>
+      <c r="E1989">
+        <v>-77.92270660400391</v>
+      </c>
+    </row>
+    <row r="1990" spans="1:5">
+      <c r="A1990" s="1" t="s">
+        <v>1992</v>
+      </c>
+      <c r="C1990">
+        <v>19.40279197692871</v>
+      </c>
+      <c r="D1990">
+        <v>-100</v>
+      </c>
+      <c r="E1990">
+        <v>17.5788402557373</v>
+      </c>
+    </row>
+    <row r="1991" spans="1:5">
+      <c r="A1991" s="1" t="s">
+        <v>1993</v>
+      </c>
+      <c r="C1991">
+        <v>2.188337564468384</v>
+      </c>
+      <c r="D1991">
+        <v>5.889395713806152</v>
+      </c>
+      <c r="E1991">
+        <v>8.623011589050293</v>
+      </c>
+    </row>
+    <row r="1992" spans="1:5">
+      <c r="A1992" s="1" t="s">
+        <v>1994</v>
+      </c>
+      <c r="C1992">
+        <v>1.177012801170349</v>
+      </c>
+      <c r="D1992">
+        <v>2.77308201789856</v>
+      </c>
+      <c r="E1992">
+        <v>4.479422569274902</v>
+      </c>
+    </row>
+    <row r="1993" spans="1:5">
+      <c r="A1993" s="1" t="s">
+        <v>1995</v>
+      </c>
+      <c r="C1993">
+        <v>-20.85583114624023</v>
+      </c>
+      <c r="D1993">
+        <v>-20.57200622558594</v>
+      </c>
+      <c r="E1993">
+        <v>-19.89276695251465</v>
+      </c>
+    </row>
+    <row r="1994" spans="1:5">
+      <c r="A1994" s="1" t="s">
+        <v>1996</v>
+      </c>
+      <c r="C1994">
+        <v>17.93227767944336</v>
+      </c>
+      <c r="D1994">
+        <v>20.84437561035156</v>
+      </c>
+      <c r="E1994">
+        <v>40.6120719909668</v>
+      </c>
+    </row>
+    <row r="1995" spans="1:5">
+      <c r="A1995" s="1" t="s">
+        <v>1997</v>
+      </c>
+      <c r="C1995">
+        <v>0.399497777223587</v>
+      </c>
+      <c r="D1995">
+        <v>3.639297723770142</v>
+      </c>
+      <c r="E1995">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="1996" spans="1:5">
+      <c r="A1996" s="1" t="s">
+        <v>1998</v>
+      </c>
+      <c r="C1996">
+        <v>9.841521263122559</v>
+      </c>
+      <c r="D1996">
+        <v>11.68402194976807</v>
+      </c>
+      <c r="E1996">
+        <v>9.311573028564453</v>
+      </c>
+    </row>
+    <row r="1997" spans="1:5">
+      <c r="A1997" s="1" t="s">
+        <v>1999</v>
+      </c>
+      <c r="C1997">
+        <v>3.434762477874756</v>
+      </c>
+      <c r="D1997">
+        <v>5.923059940338135</v>
+      </c>
+      <c r="E1997">
+        <v>7.93340015411377</v>
+      </c>
+    </row>
+    <row r="1998" spans="1:5">
+      <c r="A1998" s="1" t="s">
+        <v>2000</v>
+      </c>
+      <c r="C1998">
+        <v>3.793755292892456</v>
+      </c>
+      <c r="D1998">
+        <v>6.665188312530518</v>
+      </c>
+      <c r="E1998">
+        <v>8.342541694641113</v>
+      </c>
+    </row>
+    <row r="1999" spans="1:5">
+      <c r="A1999" s="1" t="s">
+        <v>2001</v>
+      </c>
+      <c r="C1999" t="s">
+        <v>2024</v>
+      </c>
+      <c r="D1999" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E1999" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2000" spans="1:5">
+      <c r="A2000" s="1" t="s">
+        <v>2002</v>
+      </c>
+      <c r="C2000">
+        <v>0</v>
+      </c>
+      <c r="D2000">
+        <v>0</v>
+      </c>
+      <c r="E2000">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2001" spans="1:5">
+      <c r="A2001" s="1" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C2001">
+        <v>2.583913564682007</v>
+      </c>
+      <c r="D2001">
+        <v>3.495292186737061</v>
+      </c>
+      <c r="E2001">
+        <v>4.579998970031738</v>
+      </c>
+    </row>
+    <row r="2002" spans="1:5">
+      <c r="A2002" s="1" t="s">
+        <v>2004</v>
+      </c>
+      <c r="C2002">
+        <v>11.3723611831665</v>
+      </c>
+      <c r="D2002">
+        <v>6.747061252593994</v>
+      </c>
+      <c r="E2002">
+        <v>10.55101108551025</v>
+      </c>
+    </row>
+    <row r="2003" spans="1:5">
+      <c r="A2003" s="1" t="s">
+        <v>2005</v>
+      </c>
+      <c r="C2003">
+        <v>7.819004058837891</v>
+      </c>
+      <c r="D2003">
+        <v>90.38050842285156</v>
+      </c>
+      <c r="E2003">
+        <v>5.406156063079834</v>
+      </c>
+    </row>
+    <row r="2004" spans="1:5">
+      <c r="A2004" s="1" t="s">
+        <v>2006</v>
+      </c>
+      <c r="C2004">
+        <v>11.47342491149902</v>
+      </c>
+      <c r="D2004">
+        <v>19.12232971191406</v>
+      </c>
+      <c r="E2004">
+        <v>18.26775741577148</v>
+      </c>
+    </row>
+    <row r="2005" spans="1:5">
+      <c r="A2005" s="1" t="s">
+        <v>2007</v>
+      </c>
+      <c r="C2005">
+        <v>1.28216540813446</v>
+      </c>
+      <c r="D2005">
+        <v>4.958264350891113</v>
+      </c>
+      <c r="E2005">
+        <v>-83.65345764160156</v>
+      </c>
+    </row>
+    <row r="2006" spans="1:5">
+      <c r="A2006" s="1" t="s">
+        <v>2008</v>
+      </c>
+      <c r="C2006">
+        <v>8.433977127075195</v>
+      </c>
+      <c r="D2006">
+        <v>9.899059295654297</v>
+      </c>
+      <c r="E2006">
+        <v>10.91853713989258</v>
+      </c>
+    </row>
+    <row r="2007" spans="1:5">
+      <c r="A2007" s="1" t="s">
+        <v>2009</v>
+      </c>
+      <c r="C2007">
+        <v>4.245435237884521</v>
+      </c>
+      <c r="D2007">
+        <v>3.101895809173584</v>
+      </c>
+      <c r="E2007">
+        <v>9.799628257751465</v>
+      </c>
+    </row>
+    <row r="2008" spans="1:5">
+      <c r="A2008" s="1" t="s">
+        <v>2010</v>
+      </c>
+      <c r="C2008">
+        <v>9.317231178283691</v>
+      </c>
+      <c r="D2008">
+        <v>11.17052459716797</v>
+      </c>
+      <c r="E2008">
+        <v>7.177564144134521</v>
+      </c>
+    </row>
+    <row r="2009" spans="1:5">
+      <c r="A2009" s="1" t="s">
+        <v>2011</v>
+      </c>
+      <c r="C2009">
+        <v>1090.74609375</v>
+      </c>
+      <c r="D2009">
+        <v>973.3925170898438</v>
+      </c>
+      <c r="E2009">
+        <v>885.6720581054688</v>
+      </c>
+    </row>
+    <row r="2010" spans="1:5">
+      <c r="A2010" s="1" t="s">
+        <v>2012</v>
+      </c>
+      <c r="C2010">
+        <v>350.5106811523438</v>
+      </c>
+      <c r="D2010">
+        <v>362.3034362792969</v>
+      </c>
+      <c r="E2010">
+        <v>314.7750854492188</v>
+      </c>
+    </row>
+    <row r="2011" spans="1:5">
+      <c r="A2011" s="1" t="s">
+        <v>2013</v>
+      </c>
+      <c r="C2011">
+        <v>15.91605186462402</v>
+      </c>
+      <c r="D2011">
+        <v>15.83144378662109</v>
+      </c>
+      <c r="E2011">
+        <v>15.29609203338623</v>
+      </c>
+    </row>
+    <row r="2012" spans="1:5">
+      <c r="A2012" s="1" t="s">
+        <v>2014</v>
+      </c>
+      <c r="C2012">
+        <v>10.05361270904541</v>
+      </c>
+      <c r="D2012">
+        <v>6.979473114013672</v>
+      </c>
+      <c r="E2012">
+        <v>12.2914342880249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>